<commit_message>
Work on project 1 and assignment 4
</commit_message>
<xml_diff>
--- a/Project 1/info_templat.xlsx
+++ b/Project 1/info_templat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhouzepeng/Desktop/课程/# 25 fall/DATASCI-530_Computing1 /computing_25fall/Project 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0640C435-7679-9346-ACC6-CBA6D41262D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEAFC92E-31C7-034B-8CEE-DE2C48811A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{819D12EF-4BA6-D247-B8DA-22FA2E50DE74}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Index</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -83,6 +83,18 @@
   </si>
   <si>
     <t>Production Company</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cast 1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cast 2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cast 3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -476,16 +488,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB94D6A7-32FC-5047-A4DB-3306EC6590D7}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="5" max="5" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -504,22 +518,31 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>